<commit_message>
Update Vingroup bond benchmark (secured, 8% cap) and set collateral calculator to KRW 400bn
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01JkmxWL94b2TGL1qFG2y35j
</commit_message>
<xml_diff>
--- a/output/Sunshine_vs_Vingroup_Credit_Model.xlsx
+++ b/output/Sunshine_vs_Vingroup_Credit_Model.xlsx
@@ -2000,11 +2000,11 @@
         </is>
       </c>
       <c r="B3" s="13" t="n">
-        <v>300</v>
+        <v>400</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
-          <t>Assumption: same as Vingroup Arirang deal (KRW 300bn). Replace with Sunshine's target.</t>
+          <t>Assumption: matches Vingroup Arirang deal (~KRW 400bn; board approval up to 455bn). Replace with Sunshine's target.</t>
         </is>
       </c>
     </row>
@@ -2600,22 +2600,22 @@
       </c>
       <c r="B10" s="16" t="inlineStr">
         <is>
-          <t>Is Vingroup really unsecured?</t>
+          <t>Is Vingroup secured?</t>
         </is>
       </c>
       <c r="C10" s="16" t="inlineStr">
         <is>
-          <t>Vingroup board resolutions in 2025 approve 'usage of Vingroup's assets as security for corporate bonds' for some issues.</t>
+          <t>Vingroup board resolution of 11 Aug 2026 (up to KRW 455bn, 3 years, coupon cap 8%) is reported as secured by 4 outlets; CafeF says unsecured. Pledged assets not disclosed.</t>
         </is>
       </c>
       <c r="D10" s="16" t="inlineStr">
         <is>
-          <t>The 'Vin = unsecured' premise may not hold for all Vin bonds; peer comparison must be like-for-like.</t>
+          <t>Premise 'Vin unsecured' is probably wrong; a secured Sunshine bond is in line with the benchmark. Collateral quality and priority are what differentiate.</t>
         </is>
       </c>
       <c r="E10" s="16" t="inlineStr">
         <is>
-          <t>Check the KED article / Arirang prospectus for the exact security terms.</t>
+          <t>Get the original Vingroup resolution / HOSE disclosure and the Korean offering memorandum for the security package.</t>
         </is>
       </c>
     </row>

</xml_diff>